<commit_message>
One census per plot per acquisition
</commit_message>
<xml_diff>
--- a/templates/plot_meta.xlsx
+++ b/templates/plot_meta.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10215"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10308"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/johngodlee/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/johngodlee/Library/CloudStorage/GoogleDrive-johngodlee@gmail.com/My Drive/geo-trees/PDA_processing/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2ED5CAC-D6BA-FD44-9FB8-130991A0C24C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDBA5622-FDF8-C343-BE3A-D34879FF69D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="30240" windowHeight="18960" xr2:uid="{F93C1788-238A-7A40-BC85-BA0794478508}"/>
+    <workbookView xWindow="-19200" yWindow="-14040" windowWidth="19200" windowHeight="20980" activeTab="1" xr2:uid="{F93C1788-238A-7A40-BC85-BA0794478508}"/>
   </bookViews>
   <sheets>
     <sheet name="Plot meta-data" sheetId="1" r:id="rId1"/>
@@ -37,10 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="100">
-  <si>
-    <t>Question</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="98">
   <si>
     <t>Required</t>
   </si>
@@ -57,12 +54,6 @@
     <t>Plot n</t>
   </si>
   <si>
-    <t xml:space="preserve">Provide a list of all tree inventory census dates. </t>
-  </si>
-  <si>
-    <t>Which tree inventory censuses will be contributed to GEO-TREES?</t>
-  </si>
-  <si>
     <t>Length of shortest edge of the plot (m).</t>
   </si>
   <si>
@@ -81,9 +72,6 @@
     <t>If lianas are not present, enter "NA"</t>
   </si>
   <si>
-    <t>census_date_all</t>
-  </si>
-  <si>
     <t>plot_length_m</t>
   </si>
   <si>
@@ -303,12 +291,6 @@
     <t>site_id</t>
   </si>
   <si>
-    <t>census_date_geotrees</t>
-  </si>
-  <si>
-    <t>Mid-census date for each census. Separate multiple entries with a semi-colon ";". This can be either YYYY, YYYY-MM, or YYYY-MM-DD.</t>
-  </si>
-  <si>
     <t xml:space="preserve">Elevation of the plot above International Mean sea level (m). </t>
   </si>
   <si>
@@ -337,6 +319,18 @@
   </si>
   <si>
     <t>Column</t>
+  </si>
+  <si>
+    <t>census_date</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>Mid-census date for each census. This can be either YYYY, YYYY-MM, or YYYY-MM-DD.</t>
+  </si>
+  <si>
+    <t>Census date for the plot in this acquisition</t>
   </si>
 </sst>
 </file>
@@ -778,7 +772,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A18F8DAF-594F-7549-A476-16C96F70C2E7}">
-  <dimension ref="A1:H36"/>
+  <dimension ref="A1:H35"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="19.33203125" bestFit="1" customWidth="1"/>
@@ -789,234 +783,237 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="E1" s="1" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="B2" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="D2" t="s">
-        <v>1</v>
-      </c>
       <c r="E2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F2" t="s">
         <v>2</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>3</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
         <v>4</v>
-      </c>
-      <c r="H2" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="31" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="C3" s="12" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="D3" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="51" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>7</v>
+        <v>97</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="D4" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="51" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>14</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="B6" s="9"/>
-      <c r="C6" s="9"/>
-      <c r="E6" s="10"/>
+    <row r="5" spans="1:8" s="7" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="B5" s="9"/>
+      <c r="C5" s="9"/>
+      <c r="E5" s="10"/>
+    </row>
+    <row r="6" spans="1:8" ht="17" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D6" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="7" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D7" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="17" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A8" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" s="12" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="31" x14ac:dyDescent="0.2">
+      <c r="A9" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="B9" s="12" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="68" x14ac:dyDescent="0.2">
+      <c r="A10" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="B8" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D8" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A9" s="11" t="s">
-        <v>17</v>
-      </c>
-      <c r="B9" s="12" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" ht="31" x14ac:dyDescent="0.2">
-      <c r="A10" s="11" t="s">
-        <v>18</v>
-      </c>
       <c r="B10" s="12" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" ht="68" x14ac:dyDescent="0.2">
-      <c r="A11" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="B11" s="12" t="s">
-        <v>90</v>
+        <v>84</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="51" x14ac:dyDescent="0.2">
+      <c r="A11" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>70</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" ht="51" x14ac:dyDescent="0.2">
+        <v>46</v>
+      </c>
+      <c r="D11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A12" s="6" t="s">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>74</v>
+        <v>47</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="D12" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" ht="17" x14ac:dyDescent="0.2">
-      <c r="A13" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="B13" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" s="7" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="B13" s="8"/>
+      <c r="C13" s="9"/>
+      <c r="E13" s="10"/>
+    </row>
+    <row r="14" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>48</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C14" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="C13" s="3" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="B14" s="8"/>
-      <c r="C14" s="9"/>
-      <c r="E14" s="10"/>
+      <c r="D14" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="15" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>52</v>
-      </c>
-      <c r="B15" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D15" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" ht="51" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>16</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="D16" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>17</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="D17" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>18</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="D18" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>32</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D19" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>19</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="C20" s="3" t="s">
         <v>10</v>
-      </c>
-      <c r="C15" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="D15" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" ht="34" x14ac:dyDescent="0.2">
-      <c r="A16" t="s">
-        <v>53</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C16" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="D16" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" ht="51" x14ac:dyDescent="0.2">
-      <c r="A17" t="s">
-        <v>20</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="C17" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="D17" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" ht="34" x14ac:dyDescent="0.2">
-      <c r="A18" t="s">
-        <v>21</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="C18" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="D18" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" ht="17" x14ac:dyDescent="0.2">
-      <c r="A19" t="s">
-        <v>22</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="D19" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" ht="34" x14ac:dyDescent="0.2">
-      <c r="A20" t="s">
-        <v>36</v>
-      </c>
-      <c r="B20" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="C20" s="3" t="s">
-        <v>37</v>
       </c>
       <c r="D20" t="b">
         <v>1</v>
@@ -1024,13 +1021,13 @@
     </row>
     <row r="21" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>23</v>
-      </c>
-      <c r="B21" s="3" t="s">
-        <v>82</v>
+        <v>28</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>79</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>13</v>
+        <v>29</v>
       </c>
       <c r="D21" t="b">
         <v>1</v>
@@ -1038,170 +1035,156 @@
     </row>
     <row r="22" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D22" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:5" ht="51" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
+        <v>20</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ht="68" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>27</v>
+      </c>
+      <c r="B24" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="B23" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C23" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="D23" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" ht="51" x14ac:dyDescent="0.2">
-      <c r="A24" t="s">
-        <v>24</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>56</v>
-      </c>
       <c r="C24" s="3" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" ht="68" x14ac:dyDescent="0.2">
-      <c r="A25" t="s">
-        <v>31</v>
-      </c>
-      <c r="B25" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="C25" s="3" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="B26" s="9"/>
-      <c r="C26" s="9"/>
-      <c r="E26" s="10"/>
-    </row>
-    <row r="27" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="B25" s="9"/>
+      <c r="C25" s="9"/>
+      <c r="E25" s="10"/>
+    </row>
+    <row r="26" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
+        <v>42</v>
+      </c>
+      <c r="B26" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D26" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>46</v>
-      </c>
-      <c r="B27" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="A28" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="C28" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="C27" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="D27" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" ht="34" x14ac:dyDescent="0.2">
-      <c r="A28" t="s">
-        <v>25</v>
-      </c>
-      <c r="B28" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="C28" s="3" t="s">
+    </row>
+    <row r="29" spans="1:5" ht="51" x14ac:dyDescent="0.2">
+      <c r="A29" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="A30" t="s">
+        <v>36</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="C30" s="3" t="s">
         <v>66</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" ht="34" x14ac:dyDescent="0.2">
-      <c r="A29" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="B29" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="C29" s="3" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" ht="51" x14ac:dyDescent="0.2">
-      <c r="A30" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="B30" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="C30" s="3" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" ht="34" x14ac:dyDescent="0.2">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" ht="51" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" ht="51" x14ac:dyDescent="0.2">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" ht="34" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="B34" s="4" t="s">
         <v>60</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" ht="34" x14ac:dyDescent="0.2">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>44</v>
+        <v>35</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>64</v>
+        <v>24</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="A36" t="s">
-        <v>39</v>
-      </c>
-      <c r="B36" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="C36" s="3" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
   </sheetData>
@@ -1220,22 +1203,22 @@
   <sheetData>
     <row r="1" spans="1:1" ht="34" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
     </row>
     <row r="3" spans="1:1" ht="34" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
     </row>
     <row r="5" spans="1:1" ht="34" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
     </row>
     <row r="7" spans="1:1" ht="34" x14ac:dyDescent="0.2">
       <c r="A7" s="3" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update template files to match inv. guidelines
</commit_message>
<xml_diff>
--- a/templates/plot_meta.xlsx
+++ b/templates/plot_meta.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/johngodlee/Library/CloudStorage/GoogleDrive-johngodlee@gmail.com/My Drive/geo-trees/PDA_processing/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDBA5622-FDF8-C343-BE3A-D34879FF69D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17BAB754-7B00-574F-8B1D-2A595E1E3B56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-19200" yWindow="-14040" windowWidth="19200" windowHeight="20980" activeTab="1" xr2:uid="{F93C1788-238A-7A40-BC85-BA0794478508}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="15120" windowHeight="18960" xr2:uid="{F93C1788-238A-7A40-BC85-BA0794478508}"/>
   </bookViews>
   <sheets>
     <sheet name="Plot meta-data" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="93">
   <si>
     <t>Required</t>
   </si>
@@ -54,12 +54,6 @@
     <t>Plot n</t>
   </si>
   <si>
-    <t>Length of shortest edge of the plot (m).</t>
-  </si>
-  <si>
-    <t>Length of longest edge of the plot (m).</t>
-  </si>
-  <si>
     <t>Minimum diameter threshold (cm).</t>
   </si>
   <si>
@@ -72,21 +66,6 @@
     <t>If lianas are not present, enter "NA"</t>
   </si>
   <si>
-    <t>plot_length_m</t>
-  </si>
-  <si>
-    <t>plot_width_m</t>
-  </si>
-  <si>
-    <t>plot_slope_deg</t>
-  </si>
-  <si>
-    <t>plot_aspect_deg</t>
-  </si>
-  <si>
-    <t>plot_elevation_m</t>
-  </si>
-  <si>
     <t>meas_tree_stem</t>
   </si>
   <si>
@@ -171,9 +150,6 @@
     <t>E.g. old-growth, logged, secondary, plantation.</t>
   </si>
   <si>
-    <t>treatment_ref</t>
-  </si>
-  <si>
     <t>treatment</t>
   </si>
   <si>
@@ -198,15 +174,6 @@
     <t>Link to protocol document used to measure these plots.</t>
   </si>
   <si>
-    <t xml:space="preserve"> In order of preference: (1) DOI of published protocol, (2) reference of published protocol, (3) other URL, (4) link to local file.</t>
-  </si>
-  <si>
-    <t>In order of preference: (1) DOI of published document, (2) reference of published document, (3) other URL, (4) link to local file.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Provide a link to a document describing any experimental or management treatments. </t>
-  </si>
-  <si>
     <t>If this plot ever experiences landslides, earthquakes or other earth movements, describe these phenomena.</t>
   </si>
   <si>
@@ -291,12 +258,6 @@
     <t>site_id</t>
   </si>
   <si>
-    <t xml:space="preserve">Elevation of the plot above International Mean sea level (m). </t>
-  </si>
-  <si>
-    <t>In order of preference: 1) Average of GPS readings across the plot, 2) a single GPS reading, 3) Manual lookup on topographic map, 4) NA. We can query SRTM for missing values.</t>
-  </si>
-  <si>
     <t>GEO-TREES site name.</t>
   </si>
   <si>
@@ -312,25 +273,49 @@
     <t>plot_id</t>
   </si>
   <si>
-    <t>Aspect of the plot, i.e. the direction of slope (degrees relative to grid north, 0-360).</t>
-  </si>
-  <si>
-    <t>Average slope of the plot at a scale of 20 m (degrees, 0 = flat, 90 = vertical).</t>
-  </si>
-  <si>
     <t>Column</t>
   </si>
   <si>
-    <t>census_date</t>
-  </si>
-  <si>
     <t>Description</t>
   </si>
   <si>
-    <t>Mid-census date for each census. This can be either YYYY, YYYY-MM, or YYYY-MM-DD.</t>
-  </si>
-  <si>
-    <t>Census date for the plot in this acquisition</t>
+    <t>In order of preference: (1) DOI of published protocol, (2) reference of published protocol, (3) other URL, (4) link to local file.</t>
+  </si>
+  <si>
+    <t>Describe the method used to geo-locate plot corners.</t>
+  </si>
+  <si>
+    <t>Describe the instrument used (e.g. handheld GPS, differential GNSS), measurement protocol, coordinate system.</t>
+  </si>
+  <si>
+    <t>meas_stem_loc</t>
+  </si>
+  <si>
+    <t>meas_plot_loc</t>
+  </si>
+  <si>
+    <t>Describe the method used to map stems within the plot.</t>
+  </si>
+  <si>
+    <t>Describe the measurement protocol, including the equipment used, subplot arrangement.</t>
+  </si>
+  <si>
+    <t>vegetation_type</t>
+  </si>
+  <si>
+    <t>E.g. tropical evergreen broadleaf forest, tropical deciduous broadleaf, swamp forest, open savanna.</t>
+  </si>
+  <si>
+    <t>census_id</t>
+  </si>
+  <si>
+    <t>Census ID for the plot.</t>
+  </si>
+  <si>
+    <t>E.g. "1" for the first census in the plot, "2" for the second census.</t>
+  </si>
+  <si>
+    <t>Describe the vegetation type of the plot.</t>
   </si>
 </sst>
 </file>
@@ -772,7 +757,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A18F8DAF-594F-7549-A476-16C96F70C2E7}">
-  <dimension ref="A1:H35"/>
+  <dimension ref="A1:H32"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="19.33203125" bestFit="1" customWidth="1"/>
@@ -783,18 +768,18 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="E1" s="1" t="s">
-        <v>90</v>
+        <v>77</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>93</v>
+        <v>78</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>95</v>
+        <v>79</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D2" t="s">
         <v>0</v>
@@ -814,13 +799,13 @@
     </row>
     <row r="3" spans="1:8" ht="31" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>83</v>
+        <v>72</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>86</v>
+        <v>73</v>
       </c>
       <c r="C3" s="12" t="s">
-        <v>89</v>
+        <v>76</v>
       </c>
       <c r="D3" t="b">
         <v>1</v>
@@ -828,13 +813,13 @@
     </row>
     <row r="4" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>94</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>97</v>
+        <v>89</v>
+      </c>
+      <c r="B4" s="11" t="s">
+        <v>90</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="D4" t="b">
         <v>1</v>
@@ -845,147 +830,168 @@
       <c r="C5" s="9"/>
       <c r="E5" s="10"/>
     </row>
-    <row r="6" spans="1:8" ht="17" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>12</v>
+    <row r="6" spans="1:8" ht="51" x14ac:dyDescent="0.2">
+      <c r="A6" s="6" t="s">
+        <v>19</v>
       </c>
       <c r="B6" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="D6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="17" x14ac:dyDescent="0.2">
+      <c r="A7" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" s="7" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="B8" s="8"/>
+      <c r="C8" s="9"/>
+      <c r="E8" s="10"/>
+    </row>
+    <row r="9" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>40</v>
+      </c>
+      <c r="B9" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D6" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" ht="17" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
+      <c r="C9" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D9" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>41</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="D10" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="51" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>9</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="D11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>10</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="D12" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="17" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
         <v>11</v>
       </c>
-      <c r="B7" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D7" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A8" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="B8" s="12" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" ht="31" x14ac:dyDescent="0.2">
-      <c r="A9" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="B9" s="12" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" ht="68" x14ac:dyDescent="0.2">
-      <c r="A10" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="B10" s="12" t="s">
-        <v>84</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" ht="51" x14ac:dyDescent="0.2">
-      <c r="A11" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="D11" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" ht="17" x14ac:dyDescent="0.2">
-      <c r="A12" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="B13" s="8"/>
-      <c r="C13" s="9"/>
-      <c r="E13" s="10"/>
+      <c r="B13" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="D13" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="14" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>48</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>7</v>
+        <v>25</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>66</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>51</v>
+        <v>26</v>
       </c>
       <c r="D14" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>49</v>
-      </c>
-      <c r="B15" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="C15" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C15" s="3" t="s">
-        <v>50</v>
-      </c>
       <c r="D15" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="51" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>72</v>
+        <v>22</v>
       </c>
       <c r="D16" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>74</v>
+        <v>24</v>
       </c>
       <c r="D17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:5" ht="51" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>18</v>
+        <v>84</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>76</v>
+        <v>81</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>82</v>
       </c>
       <c r="D18" t="b">
         <v>1</v>
@@ -993,198 +999,156 @@
     </row>
     <row r="19" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>32</v>
+        <v>83</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>33</v>
+        <v>86</v>
       </c>
       <c r="D19" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:5" ht="51" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>19</v>
-      </c>
-      <c r="B20" s="3" t="s">
-        <v>78</v>
+        <v>13</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>44</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="D20" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="68" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>79</v>
+        <v>27</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="D21" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" ht="17" x14ac:dyDescent="0.2">
-      <c r="A22" t="s">
-        <v>30</v>
-      </c>
-      <c r="B22" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="C22" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="D22" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" ht="51" x14ac:dyDescent="0.2">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="B22" s="9"/>
+      <c r="C22" s="9"/>
+      <c r="E22" s="10"/>
+    </row>
+    <row r="23" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>20</v>
-      </c>
-      <c r="B23" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B23" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="D23" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>87</v>
+      </c>
+      <c r="B24" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>14</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="A26" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B26" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="C23" s="3" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" ht="68" x14ac:dyDescent="0.2">
-      <c r="A24" t="s">
-        <v>27</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="C24" s="3" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="B25" s="9"/>
-      <c r="C25" s="9"/>
-      <c r="E25" s="10"/>
-    </row>
-    <row r="26" spans="1:5" ht="17" x14ac:dyDescent="0.2">
-      <c r="A26" t="s">
-        <v>42</v>
-      </c>
-      <c r="B26" s="5" t="s">
-        <v>61</v>
-      </c>
       <c r="C26" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="D26" t="b">
-        <v>1</v>
+        <v>54</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>64</v>
+        <v>48</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="34" x14ac:dyDescent="0.2">
-      <c r="A28" s="2" t="s">
+      <c r="A28" t="s">
+        <v>30</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="A29" t="s">
+        <v>31</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" ht="51" x14ac:dyDescent="0.2">
+      <c r="A30" t="s">
+        <v>32</v>
+      </c>
+      <c r="B30" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="B28" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="C28" s="3" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" ht="51" x14ac:dyDescent="0.2">
-      <c r="A29" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="B29" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="C29" s="3" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" ht="34" x14ac:dyDescent="0.2">
-      <c r="A30" t="s">
-        <v>36</v>
-      </c>
-      <c r="B30" s="4" t="s">
-        <v>59</v>
-      </c>
       <c r="C30" s="3" t="s">
-        <v>66</v>
+        <v>16</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="B31" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="C31" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="C31" s="3" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+    </row>
+    <row r="32" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>57</v>
+        <v>17</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" ht="51" x14ac:dyDescent="0.2">
-      <c r="A33" t="s">
-        <v>39</v>
-      </c>
-      <c r="B33" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="C33" s="3" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" ht="34" x14ac:dyDescent="0.2">
-      <c r="A34" t="s">
-        <v>40</v>
-      </c>
-      <c r="B34" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="C34" s="3" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="A35" t="s">
-        <v>35</v>
-      </c>
-      <c r="B35" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="C35" s="3" t="s">
-        <v>41</v>
+        <v>34</v>
       </c>
     </row>
   </sheetData>
@@ -1203,22 +1167,22 @@
   <sheetData>
     <row r="1" spans="1:1" ht="34" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
-        <v>88</v>
+        <v>75</v>
       </c>
     </row>
     <row r="3" spans="1:1" ht="34" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
-        <v>81</v>
+        <v>70</v>
       </c>
     </row>
     <row r="5" spans="1:1" ht="34" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
-        <v>82</v>
+        <v>71</v>
       </c>
     </row>
     <row r="7" spans="1:1" ht="34" x14ac:dyDescent="0.2">
       <c r="A7" s="3" t="s">
-        <v>87</v>
+        <v>74</v>
       </c>
     </row>
   </sheetData>

</xml_diff>